<commit_message>
update data and log report
</commit_message>
<xml_diff>
--- a/Data/CombatInputPanel.xlsx
+++ b/Data/CombatInputPanel.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\CombatCalculatorTest\Data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58E7B0D4-52FC-44A5-BCE8-A09D3DBFBC04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520"/>
   </bookViews>
   <sheets>
     <sheet name="CombatInputPanel" sheetId="1" r:id="rId1"/>
@@ -25,12 +19,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author/>
   </authors>
   <commentList>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="E1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -45,7 +39,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="F1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -106,7 +100,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="G1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -121,7 +115,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+    <comment ref="H1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -137,7 +131,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
+    <comment ref="I1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -152,7 +146,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="L1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -266,7 +260,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -619,7 +613,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -718,7 +712,7 @@
         <v>17</v>
       </c>
       <c r="D2" s="5">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="E2" s="5">
         <v>4</v>
@@ -1147,7 +1141,7 @@
         <v>27</v>
       </c>
       <c r="D13" s="5">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="E13" s="5">
         <v>2</v>
@@ -1202,7 +1196,7 @@
         <v>17</v>
       </c>
       <c r="D14" s="5">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="E14" s="5">
         <v>3</v>

</xml_diff>